<commit_message>
Shopify leads: batch 1 partial (US kitchen)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Inventory_Order_Automation_700_Leads.xlsx
+++ b/shopify-leads/Shopify_Inventory_Order_Automation_700_Leads.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Duplicates_Removed" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Shopify_Leads'!$A$1:$AE$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Needs_Review'!$A$1:$AE$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Shopify_Leads'!$A$1:$AE$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Needs_Review'!$A$1:$AE$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Duplicates_Removed'!$A$1:$AE$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -624,8 +624,1764 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>US-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2 Hounds Design</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://2houndsdesign.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>No-pull dog harnesses, collars and leashes</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Alisha Navarro</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Alisha</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Founder/Owner</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>woof@2houndsdesign.com</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://2houndsdesign.com/products/black-freedom-no-pull-dog-harness</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Freedom No-Pull Harness in 5/8" (XS–M) and 1" (M–XXL) widths, plus harness bundles</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>The Freedom No-Pull Harness is offered in two strap widths with overlapping Medium sizes, across many colours, plus 'BUNDLE!' listings like the 1980s and Sharky Party sets.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Variant-level low-stock alerts by width/size/colour that also update the related bundle listings and notify production.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Width x size x colour creates many variants, and bundles pull from the same harness stock; founder interview mentions own factory, so production notifications fit.</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Freedom Harness size alerts</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Hi Alisha,
+I noticed the Freedom No-Pull Harness comes in both 5/8" and 1" widths, each with its own size range, in many colours, and several prints are also sold as bundles like the Sharky Party set. That adds up to a lot of variants to watch as holiday orders pick up.
+I help Shopify stores automate inventory updates, order routing and supplier or production notifications. For example, when a specific width and size drops below a set level, your production team could receive an automatic alert and the matching bundle could update at the same time.
+Which variants are usually the first to run low for you?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>https://2houndsdesign.com/products/reflective-black-freedom-no-pull-dog-harness</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>https://2houndsdesign.com/pages/donatedecember</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE2" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>US-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Branch Basics</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://branchbasics.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Non-toxic concentrate cleaning and laundry products with refillable bottles</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Allison Evans</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Allison</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>info@branchbasics.com</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://branchbasics.com/collections/starter-kits?page=2</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Starter kits (choose refillable plastic or glass bottles); Ultimate Starter Kit with 33.8 oz Concentrate, Laundry Detergent, Oxygen Boost, Dishwasher Tablets and 4 refillable bottles</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Branch Basics starter kits let customers choose refillable plastic or glass bottles, and the Ultimate Starter Kit combines the Concentrate, Laundry Detergent, Oxygen Boost, Dishwasher Tablets and four bottles.</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Kit-component inventory sync (bottle type plus each included product) and concentrate refill reminders triggered from starter-kit orders.</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Each kit pulls from several individual SKUs and a plastic/glass bottle option, and the concentrate model drives repeat refill orders.</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Starter kit components at Branch Basics</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Hi Allison,
+I noticed your starter kits let customers pick refillable plastic or glass bottles, and the Ultimate Starter Kit pulls together the Concentrate, Laundry Detergent, Oxygen Boost, Dishwasher Tablets and four bottles.
+Since each kit depends on several separate items, a shortage of glass bottles or one product can affect the whole kit. I build Shopify automation systems for inventory updates, order processing and supplier notifications. One idea is to tie kit availability to component stock, then follow each kit order with a concentrate refill reminder timed to typical usage.
+Which part of the kit is usually hardest to keep in stock?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>https://branchbasics.com/products/ultimate-starter-kit</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>https://branchbasics.com/pages/contact</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE3" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>US-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Field Company</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://fieldcompany.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Lightweight smooth cast iron cookware</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Stephen Muscarella</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Stephen</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>help@fieldcompany.com</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://fieldcompany.com/collections/cast-iron-gifts</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Skillet sets: 3-Piece Set (No.4, No.8, No.12), 5-Piece Set, 9-Piece Set (five skillets, four lids), Starter Set No.8</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Field Company sells skillets individually and in 3-, 5- and 9-piece sets, with headquarters in New York City and production and fulfillment facilities in Indiana, Illinois and Wisconsin.</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Bundle-aware inventory sync so set availability is calculated from component skillet and lid stock across the multiple fulfillment facilities.</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Sets share the same component skillets and lids, and stock sits across several facilities; automating component-based set availability keeps listings accurate.</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Keeping Field's skillet sets in sync</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Hi Stephen,
+I noticed Field sells its skillets both on their own and in 3-, 5- and 9-piece sets, and that fulfillment runs through facilities in Indiana, Illinois and Wisconsin.
+When the same No.8 or No.12 sits inside several sets, one busy week can shift what's really available. I build Shopify automations that make inventory updates, order routing and supplier notifications easier to manage. A practical example: set availability calculated automatically from component skillet and lid counts at each facility, so a set pauses only when a part runs out.
+Are your sets tracked as their own stock today, or built from components?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>https://fieldcompany.com/products/nine-piece-cast-iron-cookware-set</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>https://fieldcompany.com/pages/contact</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE4" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>US-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Giant Dog Gear</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://giantdoggear.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Heavy-duty collars and rope leashes for large dogs</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>info@giantdoggear.com</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://shop.app/m/025mdwpgzv</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Martingale Collar with Cobra Buckle, Heavy Duty Dog Collar, Field Training Leash, 'Tiny Giant' small-dog line</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Gear is handmade in Bend, Oregon with MIL-SPEC Cobra buckles and climbing rope, and the range now spans giant-breed collars plus a 'Tiny Giant' line for small dogs.</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Component-level inventory (Cobra buckles, webbing, rope, clips) that decrements per order and triggers supplier reorder alerts.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Handmade products depend on hardware components; tracking components prevents listing items that can't be built.</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Cobra buckle stock alerts</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Hi Giant Dog Gear team,
+I liked seeing that your collars and rope leashes are handmade in Bend, Oregon with MIL-SPEC Cobra buckles and woven-core climbing rope, and that the Tiny Giant line now covers small dogs too. For handmade gear, the parts on the shelf matter as much as finished stock.
+I create Shopify automations that simplify inventory updates, order processing and supplier notifications. One example: each order deducts the buckles, webbing and rope it uses, and you get an automatic reorder alert before a component runs short ahead of the holidays.
+Do you currently track hardware separately from finished products?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>https://giantdoggear.com/products/martingale-collar-with-cobra-buckle-giant-dog-collar</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>https://giantdoggear.com/policies/contact-information</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE5" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>US-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Gracie's Doggie Delights</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://graciesdoggiedelights.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Single-ingredient freeze-dried dog and cat treats</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Grace Jagler</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Grace</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>gracie@graciesdoggiedelights.com</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Decision-maker</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://shop.app/m/graciesdoggiedelights/collections/286609146014/gracies-pet-treats</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Gracie's Pet Treats and Gracie's Kitty Delights (freeze-dried chicken breast, hearts, salmon, minnows), training treats 4oz bags, bulk bags</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Alongside the dog treat line, there is a separate Kitty Delights cat line, plus 4oz training treat bags and bulk bags of the same freeze-dried proteins.</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Link bag sizes (4oz vs bulk) to shared protein batch inventory so stock across dog, cat and bulk listings updates from one count.</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Same freeze-dried proteins appear in multiple pack sizes and lines; batch-level tracking keeps listings accurate.</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Freeze-dried batch tracking for Gracie's</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Hi Grace,
+I enjoyed browsing Gracie's Doggie Delights and saw that the freeze-dried proteins come in regular bags, 4oz training treats and bulk bags, plus the Kitty Delights line for cats. With holiday gifting coming up, keeping every bag size accurate from the same batch of chicken or salmon can take time.
+I build Shopify automation systems that make inventory updates, order processing and supplier notifications simpler. One workflow: you enter each finished batch once, and the stock for all related bag sizes adjusts automatically as orders come in.
+Would tracking by batch like that be helpful for you?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>https://graciesdoggiedelights.com/collections/all</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>https://graciesdoggiedelights.com/policies/contact-information</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE6" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>US-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Leeds Dog Supply</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://leedsdogsupply.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>California-made dog collars, leashes and accessories</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>sales@leedsdogsupply.com</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://shop.app/m/1z9cyu3bw8</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Named matching collections (Hank, Lynx, Dazey, Rover, Poncho) with collar and leash; Hank Collar from $19.95, Hank Leash $25.95</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Collars and leashes are grouped into named collections such as Hank, Lynx, Dazey, Rover and Poncho, and the brand also sells through stockists.</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Shared inventory between DTC and stockist/wholesale orders with low-stock alerts per collection pattern.</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Matching collar/leash sets per pattern plus a stockist channel means the same webbing patterns serve two order streams.</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Quick idea for the Hank Collection</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Hi Leeds Dog Supply team,
+I was browsing your named collections like Hank, Lynx and Dazey, where each pattern has a matching collar and leash made in California, and saw that you also supply stockists. When online and wholesale orders share the same patterns, it helps to see stock in one place, especially before the holidays.
+I build Shopify automation systems that simplify inventory updates, order processing and supplier notifications. One idea: stockist orders get tagged automatically, deduct from the same pattern inventory, and trigger an alert when a collection's webbing is close to running out.
+Would that kind of combined view be useful?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>https://leedsdogsupply.com/collections/hank-collection</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>https://leedsdogsupply.com/pages/stockists</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE7" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>US-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Material Kitchen</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://materialkitchen.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Modern kitchen tools, knives and cutting boards</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Eunice Byun</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Eunice</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>hello@materialkitchen.com</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://materialkitchen.com/collections/sets</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>The rePrep Set (reBoard, grippy reBoard, mini reBoard) with colour options Cool Neutral, Almost Black, Mocha, Sage (Limited Edition)</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>The rePrep Set bundles three reBoards, and add-ons come in colours including Cool Neutral, Almost Black, Mocha and a limited-edition Sage.</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Colour-level stock alerts with a limited-edition sell-through tracker, and automatic hiding or back-in-stock signup when a colour in a set runs out.</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Sets combine several boards across colourways, including a limited-edition colour, so availability depends on multiple colour SKUs at once.</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Sage limited edition stock idea</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Hi Eunice,
+I came across the rePrep Set on Material's site, with three reBoards and colour options like Cool Neutral, Almost Black, Mocha and the limited-edition Sage.
+A limited colour inside a multi-piece set is the kind of thing that can sell through faster than expected around the holidays. I help Shopify stores automate inventory updates, order processing and supplier notifications. One workflow I'd suggest: a colour-level tracker that alerts your team when Sage reaches a set threshold and switches the option to a waitlist automatically instead of leaving it to a manual check.
+How do you usually plan restocks for limited colours?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>https://materialkitchen.com/products/the-reprep-set</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>https://materialkitchen.com/pages/contact</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE8" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>US-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Meliora Cleaning Products</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://meliorameansbetter.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Plastic-free household cleaning and laundry products with refills</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Kate Jakubas</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Kate</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>info@meliorameansbetter.com</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://meliorameansbetter.com/policies/shipping-policy</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Refills collection: Laundry Powder Detergent Refill (128 HE / 64 standard loads) in multiple scents, plus Laundry Refill Bundle</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Meliora's paper box laundry powder refills are designed to refill the paper-and-steel Laundry Powder canisters and come in several scents such as unscented, lavender and lemon.</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Automated refill reminders/reorder flow triggered by canister or refill purchase date, plus scent-level stock alerts for the refill SKUs.</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Refills are a repeat purchase tied to an earlier canister order and split across scent variants; timing reminders and watching scent stock keeps the refill cycle smooth.</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Refill timing idea for Meliora</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Hi Kate,
+I was looking at Meliora's refills collection and liked how the paper box laundry powder refills are made to top up the paper-and-steel canisters, with scents from unscented to lavender and lemon.
+Refills tend to follow a predictable cycle, which makes them a good fit for automation. I set up Shopify workflows that take the manual steps out of stock updates, order handling and supplier alerts. For example, a customer who bought a canister could get a refill reminder around when the box usually runs out, while you get a heads-up if one scent is running low.
+Do most refill customers reorder on their own today?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>https://meliorameansbetter.com/collections/refills</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>https://meliorameansbetter.com/policies/shipping-policy</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE9" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>US-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Piper Loop Pets</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://piperlooppets.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>USA-made dog training treats in refillable tins and pouches</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Co-founders (Carol and Anna, surnames not verified)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>info@piper-loop.com</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://shop.app/m/piperlooppets</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026 Lil Biscuit Treat Pouches (freeze-dried meats or probiotic soft chews), refillable pocket training tins</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>The 2026 Lil Biscuit Treat Pouches collection lets customers choose freeze-dried meats or probiotic chews, alongside refillable pocket training tins.</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Refill reminder / reorder flow tied to tin purchases plus stock alerts per pouch option.</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Refillable tins imply repeat refill purchases; pouches come in two treat options to track separately.</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Refill idea for Piper Loop tins</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Hi Piper Loop Pets team,
+I came across your refillable pocket training tins and the 2026 Lil Biscuit Treat Pouches, where customers pick freeze-dried meats or probiotic soft chews. Refillable products are a nice fit for repeat orders, especially heading into the holiday season.
+I set up Shopify automations that simplify inventory updates, order processing and supplier notifications. For you, one idea is a workflow that sends a refill reminder a few weeks after a tin order, while tracking stock for each pouch option and alerting you before a flavor gets low.
+Do most customers come back for refills on their own today?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>https://piperlooppets.com/collections/2026-lil-biscuit-treat-pouches</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>https://piperlooppets.com/pages/contact</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE10" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>US-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Preen Pets</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://preenpets.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Natural USA-made dog treats and dog food</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Ron Albeg</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Ron</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>info@PreenPets.com</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://shop.app/m/preenpets</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>40+ natural dog treat varieties (jerky, bully sticks, Turkey Tendon Twists) and Whole Ingredient Dog Food (from 4 lb bag)</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Preen Pets makes over 40 varieties of natural dog treats in its Eldred, Pennsylvania kitchen and also sells a Whole Ingredient Dog Food starting at a 4 lb bag.</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Production-linked stock alerts across 40+ treat SKUs plus wholesale order routing separate from retail.</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Large in-house-made catalog and a wholesale program both draw from the same kitchen output.</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>40+ treats, one stock view</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Hi Ron,
+I noticed Preen Pets produces more than 40 natural treat varieties in your Eldred kitchen, from chicken jerky to Turkey Tendon Twists, plus the Whole Ingredient Dog Food. With retail and wholesale orders both drawing on the same production, holiday weeks can get busy.
+I build Shopify automation systems that help stores simplify inventory updates, order handling and supplier notifications. One idea: a daily low-stock summary for the kitchen that lists which treat varieties need a new batch, with wholesale orders tagged and routed separately from retail.
+Would a daily batch list like that save your team time?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>https://www.preenpets.com/collections/all</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>https://www.preenpets.com/contact/</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE11" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>US-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Sassy Woof</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://sassywoof.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Dog harnesses, collars, leashes and bundles</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Christine Chang</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Christine</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>hello@sassywoof.com</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://www.sassywoof.com/collections/dog-harnesses-adjustable</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Adjustable Harnesses (XXS–XXL, sized by neck/chest) and Harness Three Piece Bundles</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Adjustable harnesses run XXSmall to XXLarge with separate size charts per harness type, and many prints are also sold as three-piece bundles (e.g. Harry Potter bundle).</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Bundle-aware inventory sync: when one size of a harness sells out, automatically update the matching bundle variants and flag low-stock sizes before holiday demand.</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Bundles share components with single harness/collar/leash SKUs across many sizes, so stock needs to stay consistent across both listings.</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Harness bundle stock idea for Sassy Woof</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Hi Christine,
+I was looking at Sassy Woof's adjustable harnesses and noticed each print comes in sizes from XXSmall to XXLarge, with many also sold as three-piece bundles like the Harry Potter set. With the holiday season approaching, keeping single items and bundles in sync by size can get tricky.
+I build Shopify automations that simplify inventory updates, order processing and supplier notifications. One idea: when a harness size runs low, the bundle using that size updates automatically and your team gets a short restock alert listing the exact print and size.
+Would something like that be useful for your bundle lineup?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>https://www.sassywoof.com/collections/dog-bundles</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>https://www.sassywoof.com/pages/contact-us</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE12" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>US-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Stargazer Cast Iron</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://stargazercastiron.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Made-in-USA cast iron cookware</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Peter Huntley</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Peter</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>info@stargazercastiron.com</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://stargazercastiron.com/policies/terms-of-service</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Cookware collection: 10.5-inch and 12-inch cast iron skillets (each offered seasoned or bare) and 13.5-inch braiser</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Stargazer designs and manufactures its skillets in Allentown, PA, and both the 10.5-inch and 12-inch skillets come in seasoned or bare finishes.</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Per-variant (size x finish) low-stock alerts tied to production planning, with automatic notification when a seasoned or bare variant drops below a threshold.</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Each skillet size has two finish variants made in-house, so stock is split across several SKUs that depend on production runs; threshold alerts help match production to holiday demand.</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Seasoned vs bare stock alerts for Stargazer</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Hi Peter,
+I noticed Stargazer makes its skillets in Allentown and offers both the 10.5-inch and 12-inch in seasoned or bare finishes. That means every size is really two separate stock items, each tied to your own production runs.
+With holiday gifting coming up, keeping those variants balanced can matter. I build Shopify automation systems that help stores simplify inventory updates, order processing and supplier notifications. One idea: an alert that flags when a specific size and finish falls below a set level, and sends a short summary to whoever schedules seasoning or casting.
+How do you currently decide which finish to produce next?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>https://stargazercastiron.com/collections/cookware</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>https://stargazercastiron.com/pages/contact</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE13" t="n">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AE1"/>
+  <autoFilter ref="A1:AE13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -636,7 +2392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -829,8 +2585,411 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>REV-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Smithey Ironware</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://smithey.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Cast iron and carbon steel cookware</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>support@smithey.com</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://smithey.com/policies/terms-of-service</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>The Founder's 3-Piece Set (No. 8 Chef Skillet, No. 10, No. 12 Cast Iron Skillets); Set of 4 No. 6 Skillets</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Smithey offers The Founder's 3-Piece Set with the No. 8 Chef, No. 10 and No. 12 skillets, as well as a Set of 4 No. 6 Skillets.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Component-based availability for multi-skillet sets and corporate gifting order routing.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Sets reuse individual skillet SKUs and a separate corporate gifting channel exists (gifting@smithey.com).</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Skillet set stock idea for Smithey</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Hi Smithey team,
+I saw The Founder's 3-Piece Set pairs the No. 8 Chef, No. 10 and No. 12 skillets, and there's also a Set of 4 No. 6 Skillets alongside your corporate gifting program.
+When individual skillets also live inside sets and bulk gift orders, holiday demand can pull the same stock in several directions. I build Shopify automations that simplify inventory updates, order processing and supplier notifications. One workflow: set availability calculated from single-skillet counts, with large gifting orders flagged so they don't quietly drain retail stock.
+Are gifting orders handled in the same Shopify inventory as retail?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>https://smithey.com/products/the-founders-3-piece-set</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>https://smithey.com/a/faq/</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>NEEDS_REVIEW</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>US location not stated in search snippets (only an 843 phone number); likely mid-size/well-known brand; no decision maker verified.</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE2" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>REV-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Marquette Castings</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://marquettecastings.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Cast iron cookware</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>support@marquettecastings.com</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.marquettecastings.com/pages/contact</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Quick inventory idea for Marquette Castings</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Hi Marquette Castings team,
+I came across Marquette Castings while looking at independent cast iron makers, and your contact page made it easy to find the right inbox. As an independent cast iron maker, you likely see demand shift between sizes during gifting season.
+I build Shopify automation systems that help stores simplify inventory updates, order processing and supplier notifications. Ahead of the holiday season, a low-stock alert per skillet size can help plan casting runs earlier.
+How do you track stock across sizes today?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>https://www.marquettecastings.com/pages/contact</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>NEEDS_REVIEW</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>no research source URL; missing product_or_collection; missing personalized_store_observation; missing inventory_order_automation_opportunity; No verified product/collection detail and no US location statement in results (810 phone number only); email draft is generic and must be personalised before use.</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE3" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>REV-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>WanderDog Designs</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://wanderdogdesigns.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Handmade yacht rope dog leashes and collars</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>wanderdogdesigns@gmail.com</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>General inbox</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://shop.app/m/5r0y4zdh18</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Rope Slip Lead; 'Small but Mighty' custom dog leashes collection; lifetime guarantee on rope leashes/collars</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Every leash and collar is handmade from yacht rope with a lifetime guarantee, and the Small but Mighty collection offers custom leashes.</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Custom-order workflow: capture rope colour/length choices into a production queue and send automatic status updates.</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Custom handmade items need order details passed cleanly to production.</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Custom leash order flow idea</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Hi WanderDog Designs team,
+I noticed every leash and collar you make is handmade from yacht rope and backed by a lifetime guarantee, and the Small but Mighty collection offers custom leashes. Custom orders like these usually carry several details that need to reach the workbench correctly, especially as holiday orders start arriving.
+I build Shopify automations that simplify inventory updates, order processing and supplier notifications. One idea is a workflow that turns each custom order into a clear production ticket with the chosen options and sends the customer an automatic update when it ships.
+How do custom orders reach production for you today?
+Best regards,
+Oseni Ibrahim
+Shopify Automation &amp; Integration Specialist</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>https://wanderdogdesigns.com/collections/small-but-mighty</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>https://wanderdogdesigns.com/policies/refund-policy</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>PUBLICLY_LISTED</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>NEEDS_REVIEW</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>NOT_SENT</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>NO_REPLY</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>email domain not the business; US location not verified in search results; email is a Gmail address (listed on own policy pages).</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="AE4" t="n">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AE1"/>
+  <autoFilter ref="A1:AE4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>